<commit_message>
Updated Happy Desk Parent Excel File
</commit_message>
<xml_diff>
--- a/docs/Happy_Desk_Dataset/Happy_Desk_Office_Supply_Dataset.xlsx
+++ b/docs/Happy_Desk_Dataset/Happy_Desk_Office_Supply_Dataset.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f3e2a6aacfb8e2a7/Documents/Wake Tech 2022-2026/Spring 26/CSC 289 Capstone Class/Orderly/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f3e2a6aacfb8e2a7/Documents/Wake Tech 2022-2026/Spring 26/CSC 289 Capstone Class/Orderly/Data Set/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CE80AF35-016C-4B92-8CC5-847FBD8B1486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{CE80AF35-016C-4B92-8CC5-847FBD8B1486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9AFE443-AA05-4038-94FE-BC891707FD8A}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="3" xr2:uid="{4DF12D28-0ABA-484E-8B3B-DEA9606551EC}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="15552" windowHeight="18576" tabRatio="665" firstSheet="4" activeTab="5" xr2:uid="{4DF12D28-0ABA-484E-8B3B-DEA9606551EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Store List" sheetId="2" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="store #16 inventory" sheetId="1" r:id="rId3"/>
     <sheet name="store #16 dec 25 orders" sheetId="4" r:id="rId4"/>
     <sheet name="store #16 jan 26 orders" sheetId="5" r:id="rId5"/>
+    <sheet name="hopkins_order_history" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1736" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1773" uniqueCount="263">
   <si>
     <t>Product ID</t>
   </si>
@@ -826,6 +827,9 @@
   </si>
   <si>
     <t>Return Started</t>
+  </si>
+  <si>
+    <t>Hopkins attorney office order history</t>
   </si>
 </sst>
 </file>
@@ -872,7 +876,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -895,6 +899,13 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -18530,4 +18541,368 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B56EC4AA-4EF4-4CF2-AAF8-F67F12CB6986}">
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="21.109375" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" customWidth="1"/>
+    <col min="3" max="3" width="22.21875" customWidth="1"/>
+    <col min="4" max="4" width="17.88671875" customWidth="1"/>
+    <col min="5" max="5" width="13.77734375" customWidth="1"/>
+    <col min="6" max="6" width="17.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>20234901</v>
+      </c>
+      <c r="B4" s="7">
+        <v>45843</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D4" s="3">
+        <v>312.44</v>
+      </c>
+      <c r="E4" s="7">
+        <v>45845</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>20234912</v>
+      </c>
+      <c r="B5" s="7">
+        <v>45856</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D5" s="3">
+        <v>128.9</v>
+      </c>
+      <c r="E5" s="7">
+        <v>45857</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>20234927</v>
+      </c>
+      <c r="B6" s="7">
+        <v>45872</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D6" s="3">
+        <v>422.11</v>
+      </c>
+      <c r="E6" s="7">
+        <v>45874</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>20234940</v>
+      </c>
+      <c r="B7" s="7">
+        <v>45883</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D7" s="3">
+        <v>189.77</v>
+      </c>
+      <c r="E7" s="7">
+        <v>45884</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>20234958</v>
+      </c>
+      <c r="B8" s="7">
+        <v>45897</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D8" s="3">
+        <v>96.33</v>
+      </c>
+      <c r="E8" s="7">
+        <v>45898</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>20234973</v>
+      </c>
+      <c r="B9" s="7">
+        <v>45902</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D9" s="3">
+        <v>544.22</v>
+      </c>
+      <c r="E9" s="7">
+        <v>45904</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>20234988</v>
+      </c>
+      <c r="B10" s="7">
+        <v>45917</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D10" s="3">
+        <v>211.09</v>
+      </c>
+      <c r="E10" s="7">
+        <v>45918</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>20235005</v>
+      </c>
+      <c r="B11" s="7">
+        <v>45931</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D11" s="3">
+        <v>388.55</v>
+      </c>
+      <c r="E11" s="7">
+        <v>45933</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>20235016</v>
+      </c>
+      <c r="B12" s="7">
+        <v>45942</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D12" s="3">
+        <v>144.19999999999999</v>
+      </c>
+      <c r="E12" s="7">
+        <v>45943</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>20235029</v>
+      </c>
+      <c r="B13" s="7">
+        <v>45957</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D13" s="3">
+        <v>118.44</v>
+      </c>
+      <c r="E13" s="7">
+        <v>45958</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="1">
+        <v>20235041</v>
+      </c>
+      <c r="B14" s="7">
+        <v>45965</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D14" s="3">
+        <v>612.77</v>
+      </c>
+      <c r="E14" s="7">
+        <v>45967</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="1">
+        <v>20235052</v>
+      </c>
+      <c r="B15" s="7">
+        <v>45980</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D15" s="3">
+        <v>233.1</v>
+      </c>
+      <c r="E15" s="7">
+        <v>45981</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="1">
+        <v>20235001</v>
+      </c>
+      <c r="B16" s="7">
+        <v>45992</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D16" s="3">
+        <v>422.19</v>
+      </c>
+      <c r="E16" s="7">
+        <v>45994</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>20235063</v>
+      </c>
+      <c r="B17" s="7">
+        <v>46003</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D17" s="3">
+        <v>138.66</v>
+      </c>
+      <c r="E17" s="7">
+        <v>46004</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
+        <v>20235074</v>
+      </c>
+      <c r="B18" s="7">
+        <v>46013</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D18" s="3">
+        <v>119.48</v>
+      </c>
+      <c r="E18" s="7">
+        <v>46014</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>